<commit_message>
Update del nombre de Josephine
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -130,13 +130,13 @@
     <t>James Garcia</t>
   </si>
   <si>
-    <t xml:space="preserve">Josephine Snedden </t>
-  </si>
-  <si>
     <t>Lizette Aguilar-McGowen</t>
   </si>
   <si>
     <t>Raveana  Noon</t>
+  </si>
+  <si>
+    <t>Josephine Snedden</t>
   </si>
   <si>
     <t>Roseli Herrera</t>
@@ -320,7 +320,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -341,6 +341,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
@@ -678,39 +681,39 @@
   <dimension ref="A1:AG18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="17" width="33.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="18" width="33.14785714285715" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21">
@@ -1000,10 +1003,10 @@
       <c r="AG6" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="5"/>
+      <c r="B7" s="4"/>
       <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
@@ -1011,7 +1014,7 @@
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
       <c r="I7" s="5"/>
-      <c r="J7" s="4"/>
+      <c r="J7" s="5"/>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
       <c r="M7" s="6"/>
@@ -1037,7 +1040,7 @@
       <c r="AG7" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="3" t="s">
         <v>39</v>
       </c>
       <c r="B8" s="4"/>
@@ -1073,42 +1076,42 @@
       <c r="AF8" s="6"/>
       <c r="AG8" s="6"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="3" t="s">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
-      <c r="S9" s="6"/>
-      <c r="T9" s="6"/>
-      <c r="U9" s="6"/>
-      <c r="V9" s="6"/>
-      <c r="W9" s="6"/>
-      <c r="X9" s="6"/>
-      <c r="Y9" s="6"/>
-      <c r="Z9" s="6"/>
-      <c r="AA9" s="6"/>
-      <c r="AB9" s="6"/>
-      <c r="AC9" s="6"/>
-      <c r="AD9" s="6"/>
-      <c r="AE9" s="6"/>
-      <c r="AF9" s="6"/>
-      <c r="AG9" s="6"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="8"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="8"/>
+      <c r="V9" s="8"/>
+      <c r="W9" s="8"/>
+      <c r="X9" s="8"/>
+      <c r="Y9" s="8"/>
+      <c r="Z9" s="8"/>
+      <c r="AA9" s="8"/>
+      <c r="AB9" s="8"/>
+      <c r="AC9" s="8"/>
+      <c r="AD9" s="8"/>
+      <c r="AE9" s="8"/>
+      <c r="AF9" s="8"/>
+      <c r="AG9" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="7" t="s">
@@ -1185,261 +1188,261 @@
       <c r="AG11" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="20.25">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
-      <c r="O12" s="10"/>
-      <c r="P12" s="10"/>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="10"/>
-      <c r="S12" s="10"/>
-      <c r="T12" s="10"/>
-      <c r="U12" s="10"/>
-      <c r="V12" s="10"/>
-      <c r="W12" s="10"/>
-      <c r="X12" s="10"/>
-      <c r="Y12" s="10"/>
-      <c r="Z12" s="10"/>
-      <c r="AA12" s="10"/>
-      <c r="AB12" s="10"/>
-      <c r="AC12" s="10"/>
-      <c r="AD12" s="10"/>
-      <c r="AE12" s="10"/>
-      <c r="AF12" s="10"/>
-      <c r="AG12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="11"/>
+      <c r="R12" s="11"/>
+      <c r="S12" s="11"/>
+      <c r="T12" s="11"/>
+      <c r="U12" s="11"/>
+      <c r="V12" s="11"/>
+      <c r="W12" s="11"/>
+      <c r="X12" s="11"/>
+      <c r="Y12" s="11"/>
+      <c r="Z12" s="11"/>
+      <c r="AA12" s="11"/>
+      <c r="AB12" s="11"/>
+      <c r="AC12" s="11"/>
+      <c r="AD12" s="11"/>
+      <c r="AE12" s="11"/>
+      <c r="AF12" s="11"/>
+      <c r="AG12" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="20.25">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
-      <c r="O13" s="10"/>
-      <c r="P13" s="10"/>
-      <c r="Q13" s="10"/>
-      <c r="R13" s="10"/>
-      <c r="S13" s="10"/>
-      <c r="T13" s="10"/>
-      <c r="U13" s="10"/>
-      <c r="V13" s="10"/>
-      <c r="W13" s="10"/>
-      <c r="X13" s="10"/>
-      <c r="Y13" s="10"/>
-      <c r="Z13" s="10"/>
-      <c r="AA13" s="10"/>
-      <c r="AB13" s="10"/>
-      <c r="AC13" s="10"/>
-      <c r="AD13" s="10"/>
-      <c r="AE13" s="10"/>
-      <c r="AF13" s="10"/>
-      <c r="AG13" s="10"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="11"/>
+      <c r="O13" s="11"/>
+      <c r="P13" s="11"/>
+      <c r="Q13" s="11"/>
+      <c r="R13" s="11"/>
+      <c r="S13" s="11"/>
+      <c r="T13" s="11"/>
+      <c r="U13" s="11"/>
+      <c r="V13" s="11"/>
+      <c r="W13" s="11"/>
+      <c r="X13" s="11"/>
+      <c r="Y13" s="11"/>
+      <c r="Z13" s="11"/>
+      <c r="AA13" s="11"/>
+      <c r="AB13" s="11"/>
+      <c r="AC13" s="11"/>
+      <c r="AD13" s="11"/>
+      <c r="AE13" s="11"/>
+      <c r="AF13" s="11"/>
+      <c r="AG13" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
-      <c r="O14" s="10"/>
-      <c r="P14" s="10"/>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
-      <c r="T14" s="10"/>
-      <c r="U14" s="10"/>
-      <c r="V14" s="10"/>
-      <c r="W14" s="10"/>
-      <c r="X14" s="10"/>
-      <c r="Y14" s="10"/>
-      <c r="Z14" s="10"/>
-      <c r="AA14" s="10"/>
-      <c r="AB14" s="10"/>
-      <c r="AC14" s="10"/>
-      <c r="AD14" s="10"/>
-      <c r="AE14" s="10"/>
-      <c r="AF14" s="10"/>
-      <c r="AG14" s="10"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="11"/>
+      <c r="R14" s="11"/>
+      <c r="S14" s="11"/>
+      <c r="T14" s="11"/>
+      <c r="U14" s="11"/>
+      <c r="V14" s="11"/>
+      <c r="W14" s="11"/>
+      <c r="X14" s="11"/>
+      <c r="Y14" s="11"/>
+      <c r="Z14" s="11"/>
+      <c r="AA14" s="11"/>
+      <c r="AB14" s="11"/>
+      <c r="AC14" s="11"/>
+      <c r="AD14" s="11"/>
+      <c r="AE14" s="11"/>
+      <c r="AF14" s="11"/>
+      <c r="AG14" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="14"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="10"/>
-      <c r="Q15" s="10"/>
-      <c r="R15" s="10"/>
-      <c r="S15" s="10"/>
-      <c r="T15" s="10"/>
-      <c r="U15" s="10"/>
-      <c r="V15" s="10"/>
-      <c r="W15" s="10"/>
-      <c r="X15" s="10"/>
-      <c r="Y15" s="10"/>
-      <c r="Z15" s="10"/>
-      <c r="AA15" s="10"/>
-      <c r="AB15" s="10"/>
-      <c r="AC15" s="10"/>
-      <c r="AD15" s="10"/>
-      <c r="AE15" s="10"/>
-      <c r="AF15" s="10"/>
-      <c r="AG15" s="10"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="11"/>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="11"/>
+      <c r="S15" s="11"/>
+      <c r="T15" s="11"/>
+      <c r="U15" s="11"/>
+      <c r="V15" s="11"/>
+      <c r="W15" s="11"/>
+      <c r="X15" s="11"/>
+      <c r="Y15" s="11"/>
+      <c r="Z15" s="11"/>
+      <c r="AA15" s="11"/>
+      <c r="AB15" s="11"/>
+      <c r="AC15" s="11"/>
+      <c r="AD15" s="11"/>
+      <c r="AE15" s="11"/>
+      <c r="AF15" s="11"/>
+      <c r="AG15" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="10"/>
-      <c r="O16" s="10"/>
-      <c r="P16" s="10"/>
-      <c r="Q16" s="10"/>
-      <c r="R16" s="10"/>
-      <c r="S16" s="10"/>
-      <c r="T16" s="10"/>
-      <c r="U16" s="10"/>
-      <c r="V16" s="10"/>
-      <c r="W16" s="10"/>
-      <c r="X16" s="10"/>
-      <c r="Y16" s="10"/>
-      <c r="Z16" s="10"/>
-      <c r="AA16" s="10"/>
-      <c r="AB16" s="10"/>
-      <c r="AC16" s="10"/>
-      <c r="AD16" s="10"/>
-      <c r="AE16" s="10"/>
-      <c r="AF16" s="10"/>
-      <c r="AG16" s="10"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="11"/>
+      <c r="Q16" s="11"/>
+      <c r="R16" s="11"/>
+      <c r="S16" s="11"/>
+      <c r="T16" s="11"/>
+      <c r="U16" s="11"/>
+      <c r="V16" s="11"/>
+      <c r="W16" s="11"/>
+      <c r="X16" s="11"/>
+      <c r="Y16" s="11"/>
+      <c r="Z16" s="11"/>
+      <c r="AA16" s="11"/>
+      <c r="AB16" s="11"/>
+      <c r="AC16" s="11"/>
+      <c r="AD16" s="11"/>
+      <c r="AE16" s="11"/>
+      <c r="AF16" s="11"/>
+      <c r="AG16" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="20.25">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
-      <c r="O17" s="10"/>
-      <c r="P17" s="10"/>
-      <c r="Q17" s="10"/>
-      <c r="R17" s="10"/>
-      <c r="S17" s="10"/>
-      <c r="T17" s="10"/>
-      <c r="U17" s="10"/>
-      <c r="V17" s="10"/>
-      <c r="W17" s="10"/>
-      <c r="X17" s="10"/>
-      <c r="Y17" s="10"/>
-      <c r="Z17" s="10"/>
-      <c r="AA17" s="10"/>
-      <c r="AB17" s="10"/>
-      <c r="AC17" s="10"/>
-      <c r="AD17" s="10"/>
-      <c r="AE17" s="10"/>
-      <c r="AF17" s="10"/>
-      <c r="AG17" s="10"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="11"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="11"/>
+      <c r="Q17" s="11"/>
+      <c r="R17" s="11"/>
+      <c r="S17" s="11"/>
+      <c r="T17" s="11"/>
+      <c r="U17" s="11"/>
+      <c r="V17" s="11"/>
+      <c r="W17" s="11"/>
+      <c r="X17" s="11"/>
+      <c r="Y17" s="11"/>
+      <c r="Z17" s="11"/>
+      <c r="AA17" s="11"/>
+      <c r="AB17" s="11"/>
+      <c r="AC17" s="11"/>
+      <c r="AD17" s="11"/>
+      <c r="AE17" s="11"/>
+      <c r="AF17" s="11"/>
+      <c r="AG17" s="11"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
-      <c r="A18" s="15"/>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
-      <c r="N18" s="15"/>
-      <c r="O18" s="15"/>
-      <c r="P18" s="15"/>
-      <c r="Q18" s="15"/>
-      <c r="R18" s="15"/>
-      <c r="S18" s="15"/>
-      <c r="T18" s="15"/>
-      <c r="U18" s="15"/>
-      <c r="V18" s="15"/>
-      <c r="W18" s="15"/>
-      <c r="X18" s="15"/>
-      <c r="Y18" s="15"/>
-      <c r="Z18" s="15"/>
-      <c r="AA18" s="15"/>
-      <c r="AB18" s="15"/>
-      <c r="AC18" s="15"/>
-      <c r="AD18" s="15"/>
-      <c r="AE18" s="15"/>
-      <c r="AF18" s="15"/>
-      <c r="AG18" s="15"/>
+      <c r="A18" s="16"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="S18" s="16"/>
+      <c r="T18" s="16"/>
+      <c r="U18" s="16"/>
+      <c r="V18" s="16"/>
+      <c r="W18" s="16"/>
+      <c r="X18" s="16"/>
+      <c r="Y18" s="16"/>
+      <c r="Z18" s="16"/>
+      <c r="AA18" s="16"/>
+      <c r="AB18" s="16"/>
+      <c r="AC18" s="16"/>
+      <c r="AD18" s="16"/>
+      <c r="AE18" s="16"/>
+      <c r="AF18" s="16"/>
+      <c r="AG18" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>